<commit_message>
MG-504/505: cheat-meal — поля Profile + слот в меню
MG-504: Profile fields bedtime_hour, cheat_meal_interval, last_cheat_meal_date
  + миграция 0005_mg_504_profile_cheat_meal
  + ProfileSerializer/ProfileUpdateSerializer (users + family)
  + types.ts UserProfile

MG-505: cheat-meal slot
  + MenuItem.is_cheat_meal + миграция 0008_menuitem_is_cheat_meal
  + generator: helpers _mg505_is_cheat_day/_pick_cheat_slot/_mark_cheat_meal_used
  + _pick_for_role(is_cheat=True) — bypass MG-302/303/502/503 для protein
  + views.py: bulk_create + апдейт last_cheat_meal_date после генерации
  + types.ts MenuItem.is_cheat_meal

Tests: 128 passed (29 users + 13 family + 86 menu)
</commit_message>
<xml_diff>
--- a/MenuGen_Backlog.xlsx
+++ b/MenuGen_Backlog.xlsx
@@ -438,7 +438,26 @@
     <t xml:space="preserve">Спринт 4</t>
   </si>
   <si>
-    <t xml:space="preserve">Отображение меню по компонентам</t>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF006100"/>
+        <rFont val="Cambria"/>
+        <family val="0"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve">✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Отображение меню по компонентам</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">В MenuPage показывать приём пищи как карточку с 3 компонентами (зерновые / белки / овощи). У каждого свой рецепт со своей кнопкой замены.</t>
@@ -455,7 +474,26 @@
     <t xml:space="preserve">MG-402</t>
   </si>
   <si>
-    <t xml:space="preserve">Замена рецепта — фильтрация по component_role</t>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF006100"/>
+        <rFont val="Cambria"/>
+        <family val="0"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve">✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Замена рецепта — фильтрация по component_role</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">При замене рецепта в меню показывать только рецепты с тем же food_group, что и заменяемый.</t>
@@ -472,7 +510,26 @@
     <t xml:space="preserve">MG-403</t>
   </si>
   <si>
-    <t xml:space="preserve">Сводка КБЖУ за день</t>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF006100"/>
+        <rFont val="Cambria"/>
+        <family val="0"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve">✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Сводка КБЖУ за день</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">В MenuPage над каждым днём показывать суммарные КБЖУ всех приёмов и сравнение с целью пользователя (прогресс-бары).</t>
@@ -497,7 +554,26 @@
     <t xml:space="preserve">Спринт 5</t>
   </si>
   <si>
-    <t xml:space="preserve">Дополнительные поля Recipe: cooking_method, has_added_sugar, oil_tsp</t>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF006100"/>
+        <rFont val="Cambria"/>
+        <family val="0"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve">✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Дополнительные поля Recipe: cooking_method, has_added_sugar, oil_tsp</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Поля для контроля метода готовки, добавленного сахара и расхода масла.</t>
@@ -519,7 +595,26 @@
     <t xml:space="preserve">MG-502</t>
   </si>
   <si>
-    <t xml:space="preserve">Контроль масла ≤5 ч.л./день в генераторе</t>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF006100"/>
+        <rFont val="Cambria"/>
+        <family val="0"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve">✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Контроль масла ≤5 ч.л./день в генераторе</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Суммировать oil_tsp по всем рецептам дня; если &gt;5 — снижать вероятность выбора рецептов с oil_tsp&gt;1.</t>
@@ -531,7 +626,26 @@
     <t xml:space="preserve">MG-503</t>
   </si>
   <si>
-    <t xml:space="preserve">Исключение рецептов с добавленным сахаром из основных приёмов</t>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF006100"/>
+        <rFont val="Cambria"/>
+        <family val="0"/>
+        <charset val="204"/>
+      </rPr>
+      <t xml:space="preserve">✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Исключение рецептов с добавленным сахаром из основных приёмов</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">В основные приёмы (breakfast/lunch/dinner) не подставлять рецепты с has_added_sugar=True. Разрешать только в snack (как сладость, 1 раз в день).</t>
@@ -1859,7 +1973,7 @@
       <c r="D15" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" s="12" t="s">
         <v>89</v>
       </c>
       <c r="F15" s="6" t="s">
@@ -1891,7 +2005,7 @@
       <c r="D16" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" s="12" t="s">
         <v>94</v>
       </c>
       <c r="F16" s="6" t="s">
@@ -1923,7 +2037,7 @@
       <c r="D17" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" s="12" t="s">
         <v>99</v>
       </c>
       <c r="F17" s="6" t="s">
@@ -1955,7 +2069,7 @@
       <c r="D18" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E18" s="12" t="s">
         <v>107</v>
       </c>
       <c r="F18" s="6" t="s">
@@ -1987,7 +2101,7 @@
       <c r="D19" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" s="12" t="s">
         <v>112</v>
       </c>
       <c r="F19" s="6" t="s">
@@ -2019,7 +2133,7 @@
       <c r="D20" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" s="12" t="s">
         <v>116</v>
       </c>
       <c r="F20" s="6" t="s">

</xml_diff>

<commit_message>
docs: T-15 changelog + backlog (s1 recipe-repeat work)
- CHANGELOG: MG_S1ANALYZE, MG_DRINK, MG_TGIMPORT entries
- Backlog: add MG-T15 row (status 🟡, salad/snack/bakery pools still short)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DVvxSzuDV2yR9JsZysaHSr
</commit_message>
<xml_diff>
--- a/MenuGen_Backlog.xlsx
+++ b/MenuGen_Backlog.xlsx
@@ -744,7 +744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="27" min="1" max="1"/>
@@ -2055,6 +2055,56 @@
       </c>
       <c r="J24" s="43" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>MG-T15</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Backend / Data</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>🟡 Наполнить БД рецептами для s1 (борьба с повторами)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Высокая повторяемость рецептов в стратегии 1. Диагностика mg_analyze_s1_repeats показала: причина не в алгоритме, а в нехватке пула. Формула N≥d/T (min=1×d, good=4×d, great=10×d при d слотов/нед). Сделано: убраны напитки из s1 (MG_DRINK), импорт tati_cooks (MG_TGIMPORT, salad 20→32). Осталось дотянуть жёлтые пулы до good(4×спрос): salad 32→56, snack 26→56, bakery 27→28. Нужен ещё источник рецептов с КБЖУ.</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>backend/apps/menu/generator.py, backend/apps/menu/management/commands/mg_analyze_s1_repeats.py, backend/apps/recipes/management/commands/import_telegram_recipes.py</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Найти источник салатов/снеков с КБЖУ; написать парсер/импорт по образцу import_telegram_recipes; после импорта прогнать mg_seed_plate --apply, mg_backfill_recipe_products, mg_analyze_s1_repeats --runs 20 --days 7.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>MG-301, MG-302</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>